<commit_message>
feat: kafka health monitoring all 4 layers + dashboard v3.1 - DATA AGE alarm, audio alerts, producer heartbeat panel, stall watchdog, _redis_client bugfix, kafka-python in Dockerfile, MAX_INVENTORY_BTC 0.10 everywhere
</commit_message>
<xml_diff>
--- a/HFT_errors.xlsx
+++ b/HFT_errors.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7320" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7320"/>
   </bookViews>
   <sheets>
     <sheet name="History_flow" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="878" uniqueCount="785">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="790">
   <si>
     <t>This is the Framework finalized</t>
   </si>
@@ -6679,6 +6679,21 @@
   </si>
   <si>
     <t>Calculation of Information coefficient . No run due to error.</t>
+  </si>
+  <si>
+    <t>Gate calculation issue resolved. All the values will be calculated,  before the the Python engine shuts.</t>
+  </si>
+  <si>
+    <t>Incorporate Jenkins to update codes for every push 2) Validate all the Test cases for  very push and save the results.</t>
+  </si>
+  <si>
+    <t>Build 7 was showing errors</t>
+  </si>
+  <si>
+    <t>Build 15 running. Facing issue with 11 gates calculation.  Kafka producer is stopping frequently.</t>
+  </si>
+  <si>
+    <t>Uptime issues</t>
   </si>
 </sst>
 </file>
@@ -7051,7 +7066,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -7217,6 +7232,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -15882,88 +15904,115 @@
       <c r="B1055" s="15">
         <v>46129</v>
       </c>
+      <c r="C1055" s="41" t="s">
+        <v>785</v>
+      </c>
     </row>
     <row r="1056" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1056">
         <v>1055</v>
       </c>
-    </row>
-    <row r="1057" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1056" s="15">
+        <v>46130</v>
+      </c>
+      <c r="C1056" s="41" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="1057" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1057">
         <v>1056</v>
       </c>
-    </row>
-    <row r="1058" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1057" s="15">
+        <v>46131</v>
+      </c>
+      <c r="C1057" s="41" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="1058" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1058">
         <v>1057</v>
       </c>
-    </row>
-    <row r="1059" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1058" s="15">
+        <v>46132</v>
+      </c>
+      <c r="C1058" s="41" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="1059" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1059">
         <v>1058</v>
       </c>
-    </row>
-    <row r="1060" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1059" s="15">
+        <v>46133</v>
+      </c>
+      <c r="C1059" s="41" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="1060" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1060">
         <v>1059</v>
       </c>
     </row>
-    <row r="1061" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1061" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1061">
         <v>1060</v>
       </c>
     </row>
-    <row r="1062" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1062" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1062">
         <v>1061</v>
       </c>
     </row>
-    <row r="1063" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1063" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1063">
         <v>1062</v>
       </c>
     </row>
-    <row r="1064" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1064" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1064">
         <v>1063</v>
       </c>
     </row>
-    <row r="1065" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1065" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1065">
         <v>1064</v>
       </c>
     </row>
-    <row r="1066" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1066" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1066">
         <v>1065</v>
       </c>
     </row>
-    <row r="1067" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1067" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1067">
         <v>1066</v>
       </c>
     </row>
-    <row r="1068" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1068" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1068">
         <v>1067</v>
       </c>
     </row>
-    <row r="1069" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1069" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1069">
         <v>1068</v>
       </c>
     </row>
-    <row r="1070" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1070" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1070">
         <v>1069</v>
       </c>
     </row>
-    <row r="1071" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1071" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1071">
         <v>1070</v>
       </c>
     </row>
-    <row r="1072" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1072" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1072">
         <v>1071</v>
       </c>
@@ -16130,7 +16179,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -16336,10 +16385,49 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C17" s="57">
-        <f>SUM(C3:C16)</f>
-        <v>15.437999999999997</v>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="50">
+        <v>46132</v>
+      </c>
+      <c r="B15" s="52">
+        <v>170</v>
+      </c>
+      <c r="C15" s="56">
+        <f>B15/C1*100</f>
+        <v>0.16999999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="50">
+        <v>46133</v>
+      </c>
+      <c r="B16" s="52">
+        <v>218</v>
+      </c>
+      <c r="C16" s="56">
+        <f>B16/C1*100</f>
+        <v>0.218</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="59"/>
+      <c r="B17" s="60"/>
+      <c r="C17" s="61"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="59"/>
+      <c r="B18" s="60"/>
+      <c r="C18" s="61"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="59"/>
+      <c r="B19" s="60"/>
+      <c r="C19" s="61"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C20" s="57">
+        <f>SUM(C3:C19)</f>
+        <v>15.825999999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>